<commit_message>
Stabilize position manager, fix duplicate blocks, clean analyze report logging, remove pyc tracking
</commit_message>
<xml_diff>
--- a/trading_summary.xlsx
+++ b/trading_summary.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -443,7 +443,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-06 11:33:59</t>
+          <t>2026-02-06 12:59:53</t>
         </is>
       </c>
     </row>
@@ -557,45 +557,81 @@
         <v>0.15</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>mdd</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Regime</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>winrate_pct</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>avg_pct</t>
-        </is>
-      </c>
+          <t>mdd_start</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>mdd_end</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>winrate_pct</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>avg_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>winrate_pct</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>avg_pct</t>
         </is>

</xml_diff>